<commit_message>
Refactor model to formula-driven two-scenario comparison and update deck
</commit_message>
<xml_diff>
--- a/solution_zadacha2/Задача для ИИ 2 - решение.xlsx
+++ b/solution_zadacha2/Задача для ИИ 2 - решение.xlsx
@@ -118,8 +118,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="0.000"/>
-    <numFmt numFmtId="165" formatCode="0.0000"/>
+    <numFmt numFmtId="164" formatCode="0.0000"/>
+    <numFmt numFmtId="165" formatCode="0.000"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -162,7 +162,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -177,6 +177,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EEF6EE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FDEDEC"/>
       </patternFill>
     </fill>
   </fills>
@@ -206,7 +216,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" wrapText="1"/>
@@ -233,11 +243,20 @@
     <xf numFmtId="4" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -588,6 +607,132 @@
 </chartSpace>
 </file>
 
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Scenario NPV comparison</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Условие'!$C$57:$D$57</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Условие'!$C$62</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Условие'!$C$57:$D$57</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Условие'!$D$62</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Scenario</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>NPV, RUB</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
@@ -629,6 +774,28 @@
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>56</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2160000" cy="1152000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="3" name="Chart 3"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2311,7 +2478,7 @@
     <row r="23" ht="20" customHeight="1">
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>РАСЧЕТНАЯ МОДЕЛЬ (решение)</t>
+          <t>РАСЧЕТНАЯ МОДЕЛЬ (формульная, 2 сценария + сравнение)</t>
         </is>
       </c>
     </row>
@@ -2434,11 +2601,11 @@
     <row r="35" ht="20" customHeight="1">
       <c r="B35" s="10" t="inlineStr">
         <is>
-          <t>IN_capex_rub_t0</t>
+          <t>IN_capex_rub_t0_ex_vat</t>
         </is>
       </c>
       <c r="C35" s="14" t="n">
-        <v>15000000</v>
+        <v>12500000</v>
       </c>
     </row>
     <row r="36" ht="20" customHeight="1"/>
@@ -2504,23 +2671,29 @@
           <t>VAL_cash_flow</t>
         </is>
       </c>
-      <c r="D43" s="14" t="n">
-        <v>-15000000</v>
-      </c>
-      <c r="E43" s="14" t="n">
-        <v>6600000</v>
-      </c>
-      <c r="F43" s="14" t="n">
-        <v>6600000</v>
-      </c>
-      <c r="G43" s="14" t="n">
-        <v>6600000</v>
-      </c>
-      <c r="H43" s="14" t="n">
-        <v>6600000</v>
-      </c>
-      <c r="I43" s="14" t="n">
-        <v>6600000</v>
+      <c r="D43" s="14">
+        <f>-$C$35</f>
+        <v/>
+      </c>
+      <c r="E43" s="14">
+        <f>$C$42</f>
+        <v/>
+      </c>
+      <c r="F43" s="14">
+        <f>$C$42</f>
+        <v/>
+      </c>
+      <c r="G43" s="14">
+        <f>$C$42</f>
+        <v/>
+      </c>
+      <c r="H43" s="14">
+        <f>$C$42</f>
+        <v/>
+      </c>
+      <c r="I43" s="14">
+        <f>$C$42</f>
+        <v/>
       </c>
     </row>
     <row r="44" ht="20" customHeight="1">
@@ -2529,26 +2702,27 @@
           <t>VAL_discount_factor</t>
         </is>
       </c>
-      <c r="D44" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="E44" s="16">
+      <c r="D44" s="21">
+        <f>1/((1+$C$26)^D24)</f>
+        <v/>
+      </c>
+      <c r="E44" s="21">
         <f>1/((1+$C$26)^E24)</f>
         <v/>
       </c>
-      <c r="F44" s="16">
+      <c r="F44" s="21">
         <f>1/((1+$C$26)^F24)</f>
         <v/>
       </c>
-      <c r="G44" s="16">
+      <c r="G44" s="21">
         <f>1/((1+$C$26)^G24)</f>
         <v/>
       </c>
-      <c r="H44" s="16">
+      <c r="H44" s="21">
         <f>1/((1+$C$26)^H24)</f>
         <v/>
       </c>
-      <c r="I44" s="16">
+      <c r="I44" s="21">
         <f>1/((1+$C$26)^I24)</f>
         <v/>
       </c>
@@ -2622,8 +2796,9 @@
           <t>VAL_NPV</t>
         </is>
       </c>
-      <c r="C48" s="14" t="n">
-        <v>7124223.646875257</v>
+      <c r="C48" s="14">
+        <f>C62</f>
+        <v/>
       </c>
     </row>
     <row r="49" ht="20" customHeight="1">
@@ -2632,8 +2807,9 @@
           <t>VAL_IRR</t>
         </is>
       </c>
-      <c r="C49" s="11" t="n">
-        <v>0.3370160393828824</v>
+      <c r="C49" s="11">
+        <f>C63</f>
+        <v/>
       </c>
     </row>
     <row r="50" ht="20" customHeight="1">
@@ -2642,8 +2818,9 @@
           <t>VAL_DPP_years</t>
         </is>
       </c>
-      <c r="C50" s="18" t="n">
-        <v>2.98403409090909</v>
+      <c r="C50" s="18">
+        <f>C64</f>
+        <v/>
       </c>
     </row>
     <row r="51" ht="20" customHeight="1">
@@ -2652,10 +2829,9 @@
           <t>VAL_decision</t>
         </is>
       </c>
-      <c r="C51" s="12" t="inlineStr">
-        <is>
-          <t>ПРИНИМАТЬ</t>
-        </is>
+      <c r="C51" s="12">
+        <f>C65</f>
+        <v/>
       </c>
     </row>
     <row r="52" ht="20" customHeight="1">
@@ -2667,8 +2843,9 @@
           <t>VAL_price_break_even_at_freq_project</t>
         </is>
       </c>
-      <c r="C53" s="13" t="n">
-        <v>219.6428571428571</v>
+      <c r="C53" s="13">
+        <f>(($C$30*$C$32*$C$28*$C$29)-$C$34)/($C$31*$C$28*$C$29)</f>
+        <v/>
       </c>
     </row>
     <row r="54" ht="20" customHeight="1">
@@ -2677,25 +2854,215 @@
           <t>VAL_freq_break_even_at_price_project</t>
         </is>
       </c>
-      <c r="C54" s="19" t="n">
-        <v>2.196428571428572</v>
+      <c r="C54" s="22">
+        <f>(($C$30*$C$32*$C$28*$C$29)-$C$34)/($C$33*$C$28*$C$29)</f>
+        <v/>
       </c>
     </row>
     <row r="55" ht="20" customHeight="1"/>
-    <row r="56" ht="20" customHeight="1"/>
-    <row r="57" ht="20" customHeight="1"/>
-    <row r="58" ht="20" customHeight="1"/>
-    <row r="59" ht="20" customHeight="1"/>
-    <row r="60" ht="20" customHeight="1"/>
-    <row r="61" ht="20" customHeight="1"/>
-    <row r="62" ht="20" customHeight="1"/>
-    <row r="63" ht="20" customHeight="1"/>
-    <row r="64" ht="20" customHeight="1"/>
-    <row r="65" ht="20" customHeight="1"/>
+    <row r="56" ht="20" customHeight="1">
+      <c r="B56" s="8" t="inlineStr">
+        <is>
+          <t>SCENARIO_COMPARISON</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="20" customHeight="1">
+      <c r="B57" s="23" t="inlineStr">
+        <is>
+          <t>Показатель</t>
+        </is>
+      </c>
+      <c r="C57" s="23" t="inlineStr">
+        <is>
+          <t>Сценарий 1: База</t>
+        </is>
+      </c>
+      <c r="D57" s="23" t="inlineStr">
+        <is>
+          <t>Сценарий 2: Консервативный</t>
+        </is>
+      </c>
+      <c r="E57" s="23" t="inlineStr">
+        <is>
+          <t>Δ (2-1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="20" customHeight="1">
+      <c r="B58" s="24" t="inlineStr">
+        <is>
+          <t>SCN_freq_project_per_month</t>
+        </is>
+      </c>
+      <c r="C58" s="13">
+        <f>$C$31</f>
+        <v/>
+      </c>
+      <c r="D58" s="13">
+        <f>$C$31+$C$69</f>
+        <v/>
+      </c>
+      <c r="E58" s="13">
+        <f>D58-C58</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59" ht="20" customHeight="1">
+      <c r="B59" s="24" t="inlineStr">
+        <is>
+          <t>SCN_price_project_rub_per_l</t>
+        </is>
+      </c>
+      <c r="C59" s="13">
+        <f>$C$33</f>
+        <v/>
+      </c>
+      <c r="D59" s="13">
+        <f>$C$33*(1+$C$68)</f>
+        <v/>
+      </c>
+      <c r="E59" s="13">
+        <f>D59-C59</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60" ht="20" customHeight="1">
+      <c r="B60" s="24" t="inlineStr">
+        <is>
+          <t>SCN_capex_rub_t0</t>
+        </is>
+      </c>
+      <c r="C60" s="13">
+        <f>$C$35</f>
+        <v/>
+      </c>
+      <c r="D60" s="13">
+        <f>$C$35</f>
+        <v/>
+      </c>
+      <c r="E60" s="13">
+        <f>D60-C60</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61" ht="20" customHeight="1">
+      <c r="B61" s="24" t="inlineStr">
+        <is>
+          <t>SCN_annual_savings</t>
+        </is>
+      </c>
+      <c r="C61" s="13">
+        <f>(($C$30*$C$28*$C$29*$C$32)-((C58*$C$28*$C$29*C59)+$C$34))*12</f>
+        <v/>
+      </c>
+      <c r="D61" s="13">
+        <f>(($C$30*$C$28*$C$29*$C$32)-((D58*$C$28*$C$29*D59)+$C$34))*12</f>
+        <v/>
+      </c>
+      <c r="E61" s="13">
+        <f>D61-C61</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62" ht="20" customHeight="1">
+      <c r="B62" s="24" t="inlineStr">
+        <is>
+          <t>SCN_NPV</t>
+        </is>
+      </c>
+      <c r="C62" s="13">
+        <f>-C60+NPV($C$26,C61,C61,C61,C61,C61)</f>
+        <v/>
+      </c>
+      <c r="D62" s="13">
+        <f>-D60+NPV($C$26,D61,D61,D61,D61,D61)</f>
+        <v/>
+      </c>
+      <c r="E62" s="13">
+        <f>D62-C62</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63" ht="20" customHeight="1">
+      <c r="B63" s="24" t="inlineStr">
+        <is>
+          <t>SCN_IRR</t>
+        </is>
+      </c>
+      <c r="C63" s="11">
+        <f>IFERROR(IRR(CHOOSE({1,2,3,4,5,6},-C60,C61,C61,C61,C61,C61)),"N/A")</f>
+        <v/>
+      </c>
+      <c r="D63" s="11">
+        <f>IFERROR(IRR(CHOOSE({1,2,3,4,5,6},-D60,D61,D61,D61,D61,D61)),"N/A")</f>
+        <v/>
+      </c>
+      <c r="E63" s="11">
+        <f>IFERROR(D63-C63,"N/A")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64" ht="20" customHeight="1">
+      <c r="B64" s="24" t="inlineStr">
+        <is>
+          <t>SCN_DPP_years</t>
+        </is>
+      </c>
+      <c r="C64" s="18">
+        <f>IF(C61&lt;=0,"N/A",IF(NPV($C$26,C61,C61,C61,C61,C61)&lt;$C$35,"N/A",LET(c1,C61/(1+$C$26),c2,C61/(1+$C$26)^2,c3,C61/(1+$C$26)^3,c4,C61/(1+$C$26)^4,c5,C61/(1+$C$26)^5,s1,c1,s2,c1+c2,s3,c1+c2+c3,s4,c1+c2+c3+c4,IF(s1&gt;=$C$35,$C$35/c1,IF(s2&gt;=$C$35,1+($C$35-s1)/c2,IF(s3&gt;=$C$35,2+($C$35-s2)/c3,IF(s4&gt;=$C$35,3+($C$35-s3)/c4,4+($C$35-s4)/c5)))))))</f>
+        <v/>
+      </c>
+      <c r="D64" s="18">
+        <f>IF(D61&lt;=0,"N/A",IF(NPV($C$26,D61,D61,D61,D61,D61)&lt;$C$35,"N/A",LET(c1,D61/(1+$C$26),c2,D61/(1+$C$26)^2,c3,D61/(1+$C$26)^3,c4,D61/(1+$C$26)^4,c5,D61/(1+$C$26)^5,s1,c1,s2,c1+c2,s3,c1+c2+c3,s4,c1+c2+c3+c4,IF(s1&gt;=$C$35,$C$35/c1,IF(s2&gt;=$C$35,1+($C$35-s1)/c2,IF(s3&gt;=$C$35,2+($C$35-s2)/c3,IF(s4&gt;=$C$35,3+($C$35-s3)/c4,4+($C$35-s4)/c5)))))))</f>
+        <v/>
+      </c>
+      <c r="E64" s="18">
+        <f>IFERROR(D64-C64,"N/A")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65" ht="20" customHeight="1">
+      <c r="B65" s="24" t="inlineStr">
+        <is>
+          <t>SCN_decision</t>
+        </is>
+      </c>
+      <c r="C65" s="25">
+        <f>IF(AND(C62&gt;0,IFERROR(C63,0)&gt;$C$26),"ПРИНИМАТЬ","ОТКЛОНИТЬ")</f>
+        <v/>
+      </c>
+      <c r="D65" s="26">
+        <f>IF(AND(D62&gt;0,IFERROR(D63,0)&gt;$C$26),"ПРИНИМАТЬ","ОТКЛОНИТЬ")</f>
+        <v/>
+      </c>
+      <c r="E65" s="27">
+        <f>IF(C65=D65,"без изменения","разные")</f>
+        <v/>
+      </c>
+    </row>
     <row r="66" ht="20" customHeight="1"/>
     <row r="67" ht="20" customHeight="1"/>
-    <row r="68" ht="20" customHeight="1"/>
-    <row r="69" ht="20" customHeight="1"/>
+    <row r="68" ht="20" customHeight="1">
+      <c r="B68" s="10" t="inlineStr">
+        <is>
+          <t>IN_scn2_price_uplift_pct</t>
+        </is>
+      </c>
+      <c r="C68" s="11" t="n">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="69" ht="20" customHeight="1">
+      <c r="B69" s="10" t="inlineStr">
+        <is>
+          <t>IN_scn2_freq_uplift_abs</t>
+        </is>
+      </c>
+      <c r="C69" s="18" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
     <row r="70" ht="20" customHeight="1">
       <c r="B70" s="20" t="inlineStr">
         <is>
@@ -2835,7 +3202,7 @@
         </is>
       </c>
       <c r="D76" s="12" t="n">
-        <v>15000000</v>
+        <v>12500000</v>
       </c>
       <c r="E76" s="12" t="n">
         <v>0</v>
@@ -2960,7 +3327,7 @@
         </is>
       </c>
       <c r="D81" s="12" t="n">
-        <v>15000000</v>
+        <v>12500000</v>
       </c>
       <c r="E81" s="12" t="n">
         <v>0</v>
@@ -3107,108 +3474,126 @@
       <c r="B92" s="13" t="n">
         <v>180</v>
       </c>
-      <c r="C92" s="14" t="n">
-        <v>13320000</v>
-      </c>
-      <c r="D92" s="14" t="n">
-        <v>29650705.90551188</v>
-      </c>
-      <c r="E92" s="11" t="n">
-        <v>0.8466484453326599</v>
-      </c>
-      <c r="F92" s="18" t="n">
-        <v>1.339301801801801</v>
+      <c r="C92" s="14">
+        <f>(($C$30*$C$28*$C$29*$C$32)-(($C$31*$C$28*$C$29*B92)+$C$34))*12</f>
+        <v/>
+      </c>
+      <c r="D92" s="14">
+        <f>-$C$35+NPV($C$26,C92,C92,C92,C92,C92)</f>
+        <v/>
+      </c>
+      <c r="E92" s="11">
+        <f>IFERROR(IRR(CHOOSE({1,2,3,4,5,6},-$C$35,C92,C92,C92,C92,C92)),"N/A")</f>
+        <v/>
+      </c>
+      <c r="F92" s="18">
+        <f>IF(C92&lt;=0,"N/A",IF(NPV($C$26,C92,C92,C92,C92,C92)&lt;$C$35,"N/A",LET(c1,C92/(1+$C$26),c2,C92/(1+$C$26)^2,c3,C92/(1+$C$26)^3,c4,C92/(1+$C$26)^4,c5,C92/(1+$C$26)^5,s1,c1,s2,c1+c2,s3,c1+c2+c3,s4,c1+c2+c3+c4,IF(s1&gt;=$C$35,$C$35/c1,IF(s2&gt;=$C$35,1+($C$35-s1)/c2,IF(s3&gt;=$C$35,2+($C$35-s2)/c3,IF(s4&gt;=$C$35,3+($C$35-s3)/c4,4+($C$35-s4)/c5)))))))</f>
+        <v/>
       </c>
     </row>
     <row r="93" ht="20" customHeight="1">
       <c r="B93" s="13" t="n">
         <v>190</v>
       </c>
-      <c r="C93" s="14" t="n">
-        <v>9960000</v>
-      </c>
-      <c r="D93" s="14" t="n">
-        <v>18387464.77619357</v>
-      </c>
-      <c r="E93" s="11" t="n">
-        <v>0.6008424781996105</v>
-      </c>
-      <c r="F93" s="18" t="n">
-        <v>1.841716867469879</v>
+      <c r="C93" s="14">
+        <f>(($C$30*$C$28*$C$29*$C$32)-(($C$31*$C$28*$C$29*B93)+$C$34))*12</f>
+        <v/>
+      </c>
+      <c r="D93" s="14">
+        <f>-$C$35+NPV($C$26,C93,C93,C93,C93,C93)</f>
+        <v/>
+      </c>
+      <c r="E93" s="11">
+        <f>IFERROR(IRR(CHOOSE({1,2,3,4,5,6},-$C$35,C93,C93,C93,C93,C93)),"N/A")</f>
+        <v/>
+      </c>
+      <c r="F93" s="18">
+        <f>IF(C93&lt;=0,"N/A",IF(NPV($C$26,C93,C93,C93,C93,C93)&lt;$C$35,"N/A",LET(c1,C93/(1+$C$26),c2,C93/(1+$C$26)^2,c3,C93/(1+$C$26)^3,c4,C93/(1+$C$26)^4,c5,C93/(1+$C$26)^5,s1,c1,s2,c1+c2,s3,c1+c2+c3,s4,c1+c2+c3+c4,IF(s1&gt;=$C$35,$C$35/c1,IF(s2&gt;=$C$35,1+($C$35-s1)/c2,IF(s3&gt;=$C$35,2+($C$35-s2)/c3,IF(s4&gt;=$C$35,3+($C$35-s3)/c4,4+($C$35-s4)/c5)))))))</f>
+        <v/>
       </c>
     </row>
     <row r="94" ht="20" customHeight="1">
       <c r="B94" s="13" t="n">
         <v>200</v>
       </c>
-      <c r="C94" s="14" t="n">
-        <v>6600000</v>
-      </c>
-      <c r="D94" s="14" t="n">
-        <v>7124223.646875257</v>
-      </c>
-      <c r="E94" s="11" t="n">
-        <v>0.3370160393828824</v>
-      </c>
-      <c r="F94" s="18" t="n">
-        <v>2.98403409090909</v>
+      <c r="C94" s="14">
+        <f>(($C$30*$C$28*$C$29*$C$32)-(($C$31*$C$28*$C$29*B94)+$C$34))*12</f>
+        <v/>
+      </c>
+      <c r="D94" s="14">
+        <f>-$C$35+NPV($C$26,C94,C94,C94,C94,C94)</f>
+        <v/>
+      </c>
+      <c r="E94" s="11">
+        <f>IFERROR(IRR(CHOOSE({1,2,3,4,5,6},-$C$35,C94,C94,C94,C94,C94)),"N/A")</f>
+        <v/>
+      </c>
+      <c r="F94" s="18">
+        <f>IF(C94&lt;=0,"N/A",IF(NPV($C$26,C94,C94,C94,C94,C94)&lt;$C$35,"N/A",LET(c1,C94/(1+$C$26),c2,C94/(1+$C$26)^2,c3,C94/(1+$C$26)^3,c4,C94/(1+$C$26)^4,c5,C94/(1+$C$26)^5,s1,c1,s2,c1+c2,s3,c1+c2+c3,s4,c1+c2+c3+c4,IF(s1&gt;=$C$35,$C$35/c1,IF(s2&gt;=$C$35,1+($C$35-s1)/c2,IF(s3&gt;=$C$35,2+($C$35-s2)/c3,IF(s4&gt;=$C$35,3+($C$35-s3)/c4,4+($C$35-s4)/c5)))))))</f>
+        <v/>
       </c>
     </row>
     <row r="95" ht="20" customHeight="1">
       <c r="B95" s="13" t="n">
         <v>210</v>
       </c>
-      <c r="C95" s="14" t="n">
-        <v>3240000</v>
-      </c>
-      <c r="D95" s="14" t="n">
-        <v>-4139017.482443056</v>
-      </c>
-      <c r="E95" s="11" t="n">
-        <v>0.0262145642403252</v>
-      </c>
-      <c r="F95" s="18" t="n">
-        <v>8.500622368311268</v>
+      <c r="C95" s="14">
+        <f>(($C$30*$C$28*$C$29*$C$32)-(($C$31*$C$28*$C$29*B95)+$C$34))*12</f>
+        <v/>
+      </c>
+      <c r="D95" s="14">
+        <f>-$C$35+NPV($C$26,C95,C95,C95,C95,C95)</f>
+        <v/>
+      </c>
+      <c r="E95" s="11">
+        <f>IFERROR(IRR(CHOOSE({1,2,3,4,5,6},-$C$35,C95,C95,C95,C95,C95)),"N/A")</f>
+        <v/>
+      </c>
+      <c r="F95" s="18">
+        <f>IF(C95&lt;=0,"N/A",IF(NPV($C$26,C95,C95,C95,C95,C95)&lt;$C$35,"N/A",LET(c1,C95/(1+$C$26),c2,C95/(1+$C$26)^2,c3,C95/(1+$C$26)^3,c4,C95/(1+$C$26)^4,c5,C95/(1+$C$26)^5,s1,c1,s2,c1+c2,s3,c1+c2+c3,s4,c1+c2+c3+c4,IF(s1&gt;=$C$35,$C$35/c1,IF(s2&gt;=$C$35,1+($C$35-s1)/c2,IF(s3&gt;=$C$35,2+($C$35-s2)/c3,IF(s4&gt;=$C$35,3+($C$35-s3)/c4,4+($C$35-s4)/c5)))))))</f>
+        <v/>
       </c>
     </row>
     <row r="96" ht="20" customHeight="1">
       <c r="B96" s="13" t="n">
         <v>215</v>
       </c>
-      <c r="C96" s="14" t="n">
-        <v>1560000</v>
-      </c>
-      <c r="D96" s="14" t="n">
-        <v>-9770638.047102213</v>
-      </c>
-      <c r="E96" s="11" t="n">
-        <v>-0.1847005661332923</v>
-      </c>
-      <c r="F96" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+      <c r="C96" s="14">
+        <f>(($C$30*$C$28*$C$29*$C$32)-(($C$31*$C$28*$C$29*B96)+$C$34))*12</f>
+        <v/>
+      </c>
+      <c r="D96" s="14">
+        <f>-$C$35+NPV($C$26,C96,C96,C96,C96,C96)</f>
+        <v/>
+      </c>
+      <c r="E96" s="11">
+        <f>IFERROR(IRR(CHOOSE({1,2,3,4,5,6},-$C$35,C96,C96,C96,C96,C96)),"N/A")</f>
+        <v/>
+      </c>
+      <c r="F96" s="12">
+        <f>IF(C96&lt;=0,"N/A",IF(NPV($C$26,C96,C96,C96,C96,C96)&lt;$C$35,"N/A",LET(c1,C96/(1+$C$26),c2,C96/(1+$C$26)^2,c3,C96/(1+$C$26)^3,c4,C96/(1+$C$26)^4,c5,C96/(1+$C$26)^5,s1,c1,s2,c1+c2,s3,c1+c2+c3,s4,c1+c2+c3+c4,IF(s1&gt;=$C$35,$C$35/c1,IF(s2&gt;=$C$35,1+($C$35-s1)/c2,IF(s3&gt;=$C$35,2+($C$35-s2)/c3,IF(s4&gt;=$C$35,3+($C$35-s3)/c4,4+($C$35-s4)/c5)))))))</f>
+        <v/>
       </c>
     </row>
     <row r="97" ht="20" customHeight="1">
       <c r="B97" s="13" t="n">
         <v>220</v>
       </c>
-      <c r="C97" s="14" t="n">
-        <v>-120000</v>
-      </c>
-      <c r="D97" s="14" t="n">
-        <v>-15402258.61176137</v>
-      </c>
-      <c r="E97" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F97" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+      <c r="C97" s="14">
+        <f>(($C$30*$C$28*$C$29*$C$32)-(($C$31*$C$28*$C$29*B97)+$C$34))*12</f>
+        <v/>
+      </c>
+      <c r="D97" s="14">
+        <f>-$C$35+NPV($C$26,C97,C97,C97,C97,C97)</f>
+        <v/>
+      </c>
+      <c r="E97" s="12">
+        <f>IFERROR(IRR(CHOOSE({1,2,3,4,5,6},-$C$35,C97,C97,C97,C97,C97)),"N/A")</f>
+        <v/>
+      </c>
+      <c r="F97" s="12">
+        <f>IF(C97&lt;=0,"N/A",IF(NPV($C$26,C97,C97,C97,C97,C97)&lt;$C$35,"N/A",LET(c1,C97/(1+$C$26),c2,C97/(1+$C$26)^2,c3,C97/(1+$C$26)^3,c4,C97/(1+$C$26)^4,c5,C97/(1+$C$26)^5,s1,c1,s2,c1+c2,s3,c1+c2+c3,s4,c1+c2+c3+c4,IF(s1&gt;=$C$35,$C$35/c1,IF(s2&gt;=$C$35,1+($C$35-s1)/c2,IF(s3&gt;=$C$35,2+($C$35-s2)/c3,IF(s4&gt;=$C$35,3+($C$35-s3)/c4,4+($C$35-s4)/c5)))))))</f>
+        <v/>
       </c>
     </row>
     <row r="98" ht="20" customHeight="1"/>
@@ -3251,108 +3636,126 @@
       <c r="B102" s="18" t="n">
         <v>1.75</v>
       </c>
-      <c r="C102" s="14" t="n">
-        <v>15000000</v>
-      </c>
-      <c r="D102" s="14" t="n">
-        <v>35282326.47017103</v>
-      </c>
-      <c r="E102" s="11" t="n">
-        <v>0.9659482366454852</v>
-      </c>
-      <c r="F102" s="18" t="n">
-        <v>1.1725</v>
+      <c r="C102" s="14">
+        <f>(($C$30*$C$28*$C$29*$C$32)-((B102*$C$28*$C$29*$C$33)+$C$34))*12</f>
+        <v/>
+      </c>
+      <c r="D102" s="14">
+        <f>-$C$35+NPV($C$26,C102,C102,C102,C102,C102)</f>
+        <v/>
+      </c>
+      <c r="E102" s="11">
+        <f>IFERROR(IRR(CHOOSE({1,2,3,4,5,6},-$C$35,C102,C102,C102,C102,C102)),"N/A")</f>
+        <v/>
+      </c>
+      <c r="F102" s="18">
+        <f>IF(C102&lt;=0,"N/A",IF(NPV($C$26,C102,C102,C102,C102,C102)&lt;$C$35,"N/A",LET(c1,C102/(1+$C$26),c2,C102/(1+$C$26)^2,c3,C102/(1+$C$26)^3,c4,C102/(1+$C$26)^4,c5,C102/(1+$C$26)^5,s1,c1,s2,c1+c2,s3,c1+c2+c3,s4,c1+c2+c3+c4,IF(s1&gt;=$C$35,$C$35/c1,IF(s2&gt;=$C$35,1+($C$35-s1)/c2,IF(s3&gt;=$C$35,2+($C$35-s2)/c3,IF(s4&gt;=$C$35,3+($C$35-s3)/c4,4+($C$35-s4)/c5)))))))</f>
+        <v/>
       </c>
     </row>
     <row r="103" ht="20" customHeight="1">
       <c r="B103" s="18" t="n">
         <v>1.9</v>
       </c>
-      <c r="C103" s="14" t="n">
-        <v>9960000</v>
-      </c>
-      <c r="D103" s="14" t="n">
-        <v>18387464.77619357</v>
-      </c>
-      <c r="E103" s="11" t="n">
-        <v>0.6008424781996105</v>
-      </c>
-      <c r="F103" s="18" t="n">
-        <v>1.841716867469879</v>
+      <c r="C103" s="14">
+        <f>(($C$30*$C$28*$C$29*$C$32)-((B103*$C$28*$C$29*$C$33)+$C$34))*12</f>
+        <v/>
+      </c>
+      <c r="D103" s="14">
+        <f>-$C$35+NPV($C$26,C103,C103,C103,C103,C103)</f>
+        <v/>
+      </c>
+      <c r="E103" s="11">
+        <f>IFERROR(IRR(CHOOSE({1,2,3,4,5,6},-$C$35,C103,C103,C103,C103,C103)),"N/A")</f>
+        <v/>
+      </c>
+      <c r="F103" s="18">
+        <f>IF(C103&lt;=0,"N/A",IF(NPV($C$26,C103,C103,C103,C103,C103)&lt;$C$35,"N/A",LET(c1,C103/(1+$C$26),c2,C103/(1+$C$26)^2,c3,C103/(1+$C$26)^3,c4,C103/(1+$C$26)^4,c5,C103/(1+$C$26)^5,s1,c1,s2,c1+c2,s3,c1+c2+c3,s4,c1+c2+c3+c4,IF(s1&gt;=$C$35,$C$35/c1,IF(s2&gt;=$C$35,1+($C$35-s1)/c2,IF(s3&gt;=$C$35,2+($C$35-s2)/c3,IF(s4&gt;=$C$35,3+($C$35-s3)/c4,4+($C$35-s4)/c5)))))))</f>
+        <v/>
       </c>
     </row>
     <row r="104" ht="20" customHeight="1">
       <c r="B104" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="C104" s="14" t="n">
-        <v>6600000</v>
-      </c>
-      <c r="D104" s="14" t="n">
-        <v>7124223.646875257</v>
-      </c>
-      <c r="E104" s="11" t="n">
-        <v>0.3370160393828824</v>
-      </c>
-      <c r="F104" s="18" t="n">
-        <v>2.98403409090909</v>
+      <c r="C104" s="14">
+        <f>(($C$30*$C$28*$C$29*$C$32)-((B104*$C$28*$C$29*$C$33)+$C$34))*12</f>
+        <v/>
+      </c>
+      <c r="D104" s="14">
+        <f>-$C$35+NPV($C$26,C104,C104,C104,C104,C104)</f>
+        <v/>
+      </c>
+      <c r="E104" s="11">
+        <f>IFERROR(IRR(CHOOSE({1,2,3,4,5,6},-$C$35,C104,C104,C104,C104,C104)),"N/A")</f>
+        <v/>
+      </c>
+      <c r="F104" s="18">
+        <f>IF(C104&lt;=0,"N/A",IF(NPV($C$26,C104,C104,C104,C104,C104)&lt;$C$35,"N/A",LET(c1,C104/(1+$C$26),c2,C104/(1+$C$26)^2,c3,C104/(1+$C$26)^3,c4,C104/(1+$C$26)^4,c5,C104/(1+$C$26)^5,s1,c1,s2,c1+c2,s3,c1+c2+c3,s4,c1+c2+c3+c4,IF(s1&gt;=$C$35,$C$35/c1,IF(s2&gt;=$C$35,1+($C$35-s1)/c2,IF(s3&gt;=$C$35,2+($C$35-s2)/c3,IF(s4&gt;=$C$35,3+($C$35-s3)/c4,4+($C$35-s4)/c5)))))))</f>
+        <v/>
       </c>
     </row>
     <row r="105" ht="20" customHeight="1">
       <c r="B105" s="18" t="n">
         <v>2.1</v>
       </c>
-      <c r="C105" s="14" t="n">
-        <v>3240000</v>
-      </c>
-      <c r="D105" s="14" t="n">
-        <v>-4139017.482443056</v>
-      </c>
-      <c r="E105" s="11" t="n">
-        <v>0.0262145642403252</v>
-      </c>
-      <c r="F105" s="18" t="n">
-        <v>8.500622368311268</v>
+      <c r="C105" s="14">
+        <f>(($C$30*$C$28*$C$29*$C$32)-((B105*$C$28*$C$29*$C$33)+$C$34))*12</f>
+        <v/>
+      </c>
+      <c r="D105" s="14">
+        <f>-$C$35+NPV($C$26,C105,C105,C105,C105,C105)</f>
+        <v/>
+      </c>
+      <c r="E105" s="11">
+        <f>IFERROR(IRR(CHOOSE({1,2,3,4,5,6},-$C$35,C105,C105,C105,C105,C105)),"N/A")</f>
+        <v/>
+      </c>
+      <c r="F105" s="18">
+        <f>IF(C105&lt;=0,"N/A",IF(NPV($C$26,C105,C105,C105,C105,C105)&lt;$C$35,"N/A",LET(c1,C105/(1+$C$26),c2,C105/(1+$C$26)^2,c3,C105/(1+$C$26)^3,c4,C105/(1+$C$26)^4,c5,C105/(1+$C$26)^5,s1,c1,s2,c1+c2,s3,c1+c2+c3,s4,c1+c2+c3+c4,IF(s1&gt;=$C$35,$C$35/c1,IF(s2&gt;=$C$35,1+($C$35-s1)/c2,IF(s3&gt;=$C$35,2+($C$35-s2)/c3,IF(s4&gt;=$C$35,3+($C$35-s3)/c4,4+($C$35-s4)/c5)))))))</f>
+        <v/>
       </c>
     </row>
     <row r="106" ht="20" customHeight="1">
       <c r="B106" s="18" t="n">
         <v>2.15</v>
       </c>
-      <c r="C106" s="14" t="n">
-        <v>1560000</v>
-      </c>
-      <c r="D106" s="14" t="n">
-        <v>-9770638.047102213</v>
-      </c>
-      <c r="E106" s="11" t="n">
-        <v>-0.1847005661332923</v>
-      </c>
-      <c r="F106" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+      <c r="C106" s="14">
+        <f>(($C$30*$C$28*$C$29*$C$32)-((B106*$C$28*$C$29*$C$33)+$C$34))*12</f>
+        <v/>
+      </c>
+      <c r="D106" s="14">
+        <f>-$C$35+NPV($C$26,C106,C106,C106,C106,C106)</f>
+        <v/>
+      </c>
+      <c r="E106" s="11">
+        <f>IFERROR(IRR(CHOOSE({1,2,3,4,5,6},-$C$35,C106,C106,C106,C106,C106)),"N/A")</f>
+        <v/>
+      </c>
+      <c r="F106" s="12">
+        <f>IF(C106&lt;=0,"N/A",IF(NPV($C$26,C106,C106,C106,C106,C106)&lt;$C$35,"N/A",LET(c1,C106/(1+$C$26),c2,C106/(1+$C$26)^2,c3,C106/(1+$C$26)^3,c4,C106/(1+$C$26)^4,c5,C106/(1+$C$26)^5,s1,c1,s2,c1+c2,s3,c1+c2+c3,s4,c1+c2+c3+c4,IF(s1&gt;=$C$35,$C$35/c1,IF(s2&gt;=$C$35,1+($C$35-s1)/c2,IF(s3&gt;=$C$35,2+($C$35-s2)/c3,IF(s4&gt;=$C$35,3+($C$35-s3)/c4,4+($C$35-s4)/c5)))))))</f>
+        <v/>
       </c>
     </row>
     <row r="107" ht="20" customHeight="1">
       <c r="B107" s="18" t="n">
         <v>2.25</v>
       </c>
-      <c r="C107" s="14" t="n">
-        <v>-1800000</v>
-      </c>
-      <c r="D107" s="14" t="n">
-        <v>-21033879.17642052</v>
-      </c>
-      <c r="E107" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F107" s="12" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+      <c r="C107" s="14">
+        <f>(($C$30*$C$28*$C$29*$C$32)-((B107*$C$28*$C$29*$C$33)+$C$34))*12</f>
+        <v/>
+      </c>
+      <c r="D107" s="14">
+        <f>-$C$35+NPV($C$26,C107,C107,C107,C107,C107)</f>
+        <v/>
+      </c>
+      <c r="E107" s="12">
+        <f>IFERROR(IRR(CHOOSE({1,2,3,4,5,6},-$C$35,C107,C107,C107,C107,C107)),"N/A")</f>
+        <v/>
+      </c>
+      <c r="F107" s="12">
+        <f>IF(C107&lt;=0,"N/A",IF(NPV($C$26,C107,C107,C107,C107,C107)&lt;$C$35,"N/A",LET(c1,C107/(1+$C$26),c2,C107/(1+$C$26)^2,c3,C107/(1+$C$26)^3,c4,C107/(1+$C$26)^4,c5,C107/(1+$C$26)^5,s1,c1,s2,c1+c2,s3,c1+c2+c3,s4,c1+c2+c3+c4,IF(s1&gt;=$C$35,$C$35/c1,IF(s2&gt;=$C$35,1+($C$35-s1)/c2,IF(s3&gt;=$C$35,2+($C$35-s2)/c3,IF(s4&gt;=$C$35,3+($C$35-s3)/c4,4+($C$35-s4)/c5)))))))</f>
+        <v/>
       </c>
     </row>
     <row r="108" ht="20" customHeight="1"/>
@@ -3420,20 +3823,25 @@
       <c r="D114" s="12" t="n">
         <v>2.15</v>
       </c>
-      <c r="E114" s="14" t="n">
-        <v>35282326.47017103</v>
-      </c>
-      <c r="F114" s="14" t="n">
-        <v>-9770638.047102213</v>
-      </c>
-      <c r="G114" s="14" t="n">
-        <v>28158102.82329578</v>
-      </c>
-      <c r="H114" s="14" t="n">
-        <v>-16894861.69397747</v>
-      </c>
-      <c r="I114" s="14" t="n">
-        <v>45052964.51727325</v>
+      <c r="E114" s="14">
+        <f>INDEX($D$102:$D$107,MATCH(C114,$B$102:$B$107,0))</f>
+        <v/>
+      </c>
+      <c r="F114" s="14">
+        <f>INDEX($D$102:$D$107,MATCH(D114,$B$102:$B$107,0))</f>
+        <v/>
+      </c>
+      <c r="G114" s="14">
+        <f>E114-$C$48</f>
+        <v/>
+      </c>
+      <c r="H114" s="14">
+        <f>F114-$C$48</f>
+        <v/>
+      </c>
+      <c r="I114" s="14">
+        <f>ABS(F114-E114)</f>
+        <v/>
       </c>
     </row>
     <row r="115" ht="20" customHeight="1">
@@ -3448,20 +3856,25 @@
       <c r="D115" s="12" t="n">
         <v>215</v>
       </c>
-      <c r="E115" s="14" t="n">
-        <v>29650705.90551188</v>
-      </c>
-      <c r="F115" s="14" t="n">
-        <v>-9770638.047102213</v>
-      </c>
-      <c r="G115" s="14" t="n">
-        <v>22526482.25863662</v>
-      </c>
-      <c r="H115" s="14" t="n">
-        <v>-16894861.69397747</v>
-      </c>
-      <c r="I115" s="14" t="n">
-        <v>39421343.9526141</v>
+      <c r="E115" s="14">
+        <f>INDEX($D$92:$D$97,MATCH(C115,$B$92:$B$97,0))</f>
+        <v/>
+      </c>
+      <c r="F115" s="14">
+        <f>INDEX($D$92:$D$97,MATCH(D115,$B$92:$B$97,0))</f>
+        <v/>
+      </c>
+      <c r="G115" s="14">
+        <f>E115-$C$48</f>
+        <v/>
+      </c>
+      <c r="H115" s="14">
+        <f>F115-$C$48</f>
+        <v/>
+      </c>
+      <c r="I115" s="14">
+        <f>ABS(F115-E115)</f>
+        <v/>
       </c>
     </row>
     <row r="116" ht="20" customHeight="1"/>
@@ -3527,20 +3940,25 @@
       <c r="D120" s="12" t="n">
         <v>2.15</v>
       </c>
-      <c r="E120" s="11" t="n">
-        <v>0.9659482366454852</v>
-      </c>
-      <c r="F120" s="11" t="n">
-        <v>-0.1847005661332923</v>
-      </c>
-      <c r="G120" s="11" t="n">
-        <v>0.6289321972626029</v>
-      </c>
-      <c r="H120" s="11" t="n">
-        <v>-0.5217166055161746</v>
-      </c>
-      <c r="I120" s="11" t="n">
-        <v>1.150648802778778</v>
+      <c r="E120" s="11">
+        <f>INDEX($E$102:$E$107,MATCH(C120,$B$102:$B$107,0))</f>
+        <v/>
+      </c>
+      <c r="F120" s="11">
+        <f>INDEX($E$102:$E$107,MATCH(D120,$B$102:$B$107,0))</f>
+        <v/>
+      </c>
+      <c r="G120" s="11">
+        <f>IFERROR(E120-$C$49,"N/A")</f>
+        <v/>
+      </c>
+      <c r="H120" s="11">
+        <f>IFERROR(F120-$C$49,"N/A")</f>
+        <v/>
+      </c>
+      <c r="I120" s="11">
+        <f>IFERROR(ABS(F120-E120),"N/A")</f>
+        <v/>
       </c>
     </row>
     <row r="121" ht="20" customHeight="1">
@@ -3555,20 +3973,25 @@
       <c r="D121" s="12" t="n">
         <v>215</v>
       </c>
-      <c r="E121" s="11" t="n">
-        <v>0.8466484453326599</v>
-      </c>
-      <c r="F121" s="11" t="n">
-        <v>-0.1847005661332923</v>
-      </c>
-      <c r="G121" s="11" t="n">
-        <v>0.5096324059497775</v>
-      </c>
-      <c r="H121" s="11" t="n">
-        <v>-0.5217166055161746</v>
-      </c>
-      <c r="I121" s="11" t="n">
-        <v>1.031349011465952</v>
+      <c r="E121" s="11">
+        <f>INDEX($E$92:$E$97,MATCH(C121,$B$92:$B$97,0))</f>
+        <v/>
+      </c>
+      <c r="F121" s="11">
+        <f>INDEX($E$92:$E$97,MATCH(D121,$B$92:$B$97,0))</f>
+        <v/>
+      </c>
+      <c r="G121" s="11">
+        <f>IFERROR(E121-$C$49,"N/A")</f>
+        <v/>
+      </c>
+      <c r="H121" s="11">
+        <f>IFERROR(F121-$C$49,"N/A")</f>
+        <v/>
+      </c>
+      <c r="I121" s="11">
+        <f>IFERROR(ABS(F121-E121),"N/A")</f>
+        <v/>
       </c>
     </row>
     <row r="122" ht="20" customHeight="1"/>

</xml_diff>